<commit_message>
Completed basic Discount function
Computes a discount of 20% from 2 inputs: Quantity, Price. If Quantity is greater than 25, apply discount.
</commit_message>
<xml_diff>
--- a/Excel-VBA-Start.xlsx
+++ b/Excel-VBA-Start.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Michael Q\Desktop\Online Course Dev\Flodesk YT Start Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\belin\Documents\CMPT310_A2\VBA_Learning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13596C26-62D1-4FFC-8D42-995A2168DFBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EEEE660-DD8D-4B44-B3E1-7D741E9E9F27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="15260" xr2:uid="{107DEBDB-C5C3-F842-80B8-32945E357030}"/>
+    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" activeTab="1" xr2:uid="{107DEBDB-C5C3-F842-80B8-32945E357030}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover Page" sheetId="3" r:id="rId1"/>
@@ -35,6 +35,28 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -218,8 +240,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -472,7 +494,7 @@
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -485,8 +507,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -598,9 +620,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -638,7 +660,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -744,7 +766,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -886,7 +908,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -896,105 +918,105 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFEA2472-6E87-443E-AC2B-8371A6CD9329}">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="B4:D19"/>
-  <sheetFormatPr defaultColWidth="9.5" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.5" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.5" style="12"/>
-    <col min="2" max="2" width="7.33203125" style="12" customWidth="1"/>
+    <col min="2" max="2" width="7.375" style="12" customWidth="1"/>
     <col min="3" max="3" width="96.75" style="12" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.25" style="12" customWidth="1"/>
     <col min="5" max="16384" width="9.5" style="12"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:4" ht="54" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:4" ht="54" x14ac:dyDescent="0.25">
       <c r="B4" s="9"/>
       <c r="C4" s="10" t="s">
         <v>44</v>
       </c>
       <c r="D4" s="11"/>
     </row>
-    <row r="5" spans="2:4" ht="64" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:4" ht="64.5" x14ac:dyDescent="0.25">
       <c r="B5" s="13"/>
       <c r="C5" s="14"/>
       <c r="D5" s="15"/>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="13"/>
       <c r="C6" s="16"/>
       <c r="D6" s="15"/>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="13"/>
       <c r="C7" s="16"/>
       <c r="D7" s="15"/>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="13"/>
       <c r="C8" s="16"/>
       <c r="D8" s="15"/>
     </row>
-    <row r="9" spans="2:4" s="20" customFormat="1" ht="21" x14ac:dyDescent="0.5">
+    <row r="9" spans="2:4" s="20" customFormat="1" ht="21" x14ac:dyDescent="0.35">
       <c r="B9" s="17"/>
       <c r="C9" s="18" t="s">
         <v>45</v>
       </c>
       <c r="D9" s="19"/>
     </row>
-    <row r="10" spans="2:4" s="20" customFormat="1" ht="21" x14ac:dyDescent="0.5">
+    <row r="10" spans="2:4" s="20" customFormat="1" ht="21" x14ac:dyDescent="0.35">
       <c r="B10" s="17"/>
       <c r="C10" s="21"/>
       <c r="D10" s="19"/>
     </row>
-    <row r="11" spans="2:4" s="25" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:4" s="25" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="22"/>
       <c r="C11" s="23" t="s">
         <v>43</v>
       </c>
       <c r="D11" s="24"/>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="13"/>
       <c r="C12" s="16"/>
       <c r="D12" s="15"/>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="13"/>
       <c r="C13" s="16"/>
       <c r="D13" s="15"/>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" s="13"/>
       <c r="C14" s="16"/>
       <c r="D14" s="15"/>
     </row>
-    <row r="15" spans="2:4" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B15" s="13"/>
       <c r="C15" s="26" t="s">
         <v>39</v>
       </c>
       <c r="D15" s="15"/>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="13"/>
       <c r="C16" s="27" t="s">
         <v>40</v>
       </c>
       <c r="D16" s="15"/>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="13"/>
       <c r="C17" s="16" t="s">
         <v>41</v>
       </c>
       <c r="D17" s="15"/>
     </row>
-    <row r="18" spans="2:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:4" ht="30" x14ac:dyDescent="0.25">
       <c r="B18" s="13"/>
       <c r="C18" s="28" t="s">
         <v>42</v>
       </c>
       <c r="D18" s="15"/>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B19" s="29"/>
       <c r="C19" s="30"/>
       <c r="D19" s="31"/>
@@ -1014,16 +1036,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A90BD485-ADB2-3744-A527-D8EE6B9EE875}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="B2:H23"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
-    <col min="2" max="2" width="9.33203125" customWidth="1"/>
+    <col min="2" max="2" width="9.375" customWidth="1"/>
     <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.6640625" customWidth="1"/>
+    <col min="5" max="5" width="9.625" customWidth="1"/>
     <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="2" spans="2:8" ht="21" x14ac:dyDescent="0.35">
       <c r="B2" s="5" t="s">
         <v>37</v>
       </c>
@@ -1034,12 +1056,12 @@
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="7" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="8" t="s">
         <v>2</v>
       </c>
@@ -1062,7 +1084,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="1">
         <v>11280</v>
       </c>
@@ -1078,13 +1100,16 @@
       <c r="F6" s="3">
         <v>30000</v>
       </c>
-      <c r="G6" s="3"/>
+      <c r="G6" s="3" cm="1">
+        <f t="array" ref="G6">Discount(E6, F6)</f>
+        <v>0</v>
+      </c>
       <c r="H6" s="4">
         <f>E6*F6-G6</f>
         <v>450000</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="1">
         <f>B6+1</f>
         <v>11281</v>
@@ -1101,13 +1126,16 @@
       <c r="F7" s="3">
         <v>25000</v>
       </c>
-      <c r="G7" s="3"/>
+      <c r="G7" s="3" cm="1">
+        <f t="array" ref="G7">Discount(E7, F7)</f>
+        <v>0</v>
+      </c>
       <c r="H7" s="4">
         <f t="shared" ref="H7:H23" si="0">E7*F7-G7</f>
         <v>250000</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="1">
         <f t="shared" ref="B8:B23" si="1">B7+1</f>
         <v>11282</v>
@@ -1124,13 +1152,16 @@
       <c r="F8" s="3">
         <v>28000</v>
       </c>
-      <c r="G8" s="3"/>
+      <c r="G8" s="3" cm="1">
+        <f t="array" ref="G8">Discount(E8, F8)</f>
+        <v>840000</v>
+      </c>
       <c r="H8" s="4">
         <f t="shared" si="0"/>
-        <v>4200000</v>
-      </c>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
+        <v>3360000</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="1">
         <f t="shared" si="1"/>
         <v>11283</v>
@@ -1147,13 +1178,16 @@
       <c r="F9" s="3">
         <v>30000</v>
       </c>
-      <c r="G9" s="3"/>
+      <c r="G9" s="3" cm="1">
+        <f t="array" ref="G9">Discount(E9, F9)</f>
+        <v>0</v>
+      </c>
       <c r="H9" s="4">
         <f t="shared" si="0"/>
         <v>360000</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="1">
         <f t="shared" si="1"/>
         <v>11284</v>
@@ -1170,13 +1204,16 @@
       <c r="F10" s="3">
         <v>30000</v>
       </c>
-      <c r="G10" s="3"/>
+      <c r="G10" s="3" cm="1">
+        <f t="array" ref="G10">Discount(E10, F10)</f>
+        <v>0</v>
+      </c>
       <c r="H10" s="4">
         <f t="shared" si="0"/>
         <v>600000</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="1">
         <f t="shared" si="1"/>
         <v>11285</v>
@@ -1193,13 +1230,16 @@
       <c r="F11" s="3">
         <v>26000</v>
       </c>
-      <c r="G11" s="3"/>
+      <c r="G11" s="3" cm="1">
+        <f t="array" ref="G11">Discount(E11, F11)</f>
+        <v>0</v>
+      </c>
       <c r="H11" s="4">
         <f t="shared" si="0"/>
         <v>520000</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" s="1">
         <f t="shared" si="1"/>
         <v>11286</v>
@@ -1216,13 +1256,16 @@
       <c r="F12" s="3">
         <v>30000</v>
       </c>
-      <c r="G12" s="3"/>
+      <c r="G12" s="3" cm="1">
+        <f t="array" ref="G12">Discount(E12, F12)</f>
+        <v>0</v>
+      </c>
       <c r="H12" s="4">
         <f t="shared" si="0"/>
         <v>60000</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="1">
         <f t="shared" si="1"/>
         <v>11287</v>
@@ -1239,13 +1282,16 @@
       <c r="F13" s="3">
         <v>35000</v>
       </c>
-      <c r="G13" s="3"/>
+      <c r="G13" s="3" cm="1">
+        <f t="array" ref="G13">Discount(E13, F13)</f>
+        <v>0</v>
+      </c>
       <c r="H13" s="4">
         <f t="shared" si="0"/>
         <v>175000</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" s="1">
         <f t="shared" si="1"/>
         <v>11288</v>
@@ -1262,13 +1308,16 @@
       <c r="F14" s="3">
         <v>30000</v>
       </c>
-      <c r="G14" s="3"/>
+      <c r="G14" s="3" cm="1">
+        <f t="array" ref="G14">Discount(E14, F14)</f>
+        <v>480000</v>
+      </c>
       <c r="H14" s="4">
         <f t="shared" si="0"/>
-        <v>2400000</v>
-      </c>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
+        <v>1920000</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="1">
         <f t="shared" si="1"/>
         <v>11289</v>
@@ -1285,13 +1334,16 @@
       <c r="F15" s="3">
         <v>26000</v>
       </c>
-      <c r="G15" s="3"/>
+      <c r="G15" s="3" cm="1">
+        <f t="array" ref="G15">Discount(E15, F15)</f>
+        <v>520000</v>
+      </c>
       <c r="H15" s="4">
         <f t="shared" si="0"/>
-        <v>2600000</v>
-      </c>
-    </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
+        <v>2080000</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16" s="1">
         <f t="shared" si="1"/>
         <v>11290</v>
@@ -1308,13 +1360,16 @@
       <c r="F16" s="3">
         <v>35000</v>
       </c>
-      <c r="G16" s="3"/>
+      <c r="G16" s="3" cm="1">
+        <f t="array" ref="G16">Discount(E16, F16)</f>
+        <v>0</v>
+      </c>
       <c r="H16" s="4">
         <f t="shared" si="0"/>
         <v>700000</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="1">
         <f t="shared" si="1"/>
         <v>11291</v>
@@ -1331,13 +1386,16 @@
       <c r="F17" s="3">
         <v>40000</v>
       </c>
-      <c r="G17" s="3"/>
+      <c r="G17" s="3" cm="1">
+        <f t="array" ref="G17">Discount(E17, F17)</f>
+        <v>0</v>
+      </c>
       <c r="H17" s="4">
-        <f t="shared" si="0"/>
+        <f>E17*F17-G17</f>
         <v>1000000</v>
       </c>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="1">
         <f t="shared" si="1"/>
         <v>11292</v>
@@ -1354,13 +1412,16 @@
       <c r="F18" s="3">
         <v>28000</v>
       </c>
-      <c r="G18" s="3"/>
+      <c r="G18" s="3" cm="1">
+        <f t="array" ref="G18">Discount(E18, F18)</f>
+        <v>0</v>
+      </c>
       <c r="H18" s="4">
         <f t="shared" si="0"/>
         <v>280000</v>
       </c>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="1">
         <f t="shared" si="1"/>
         <v>11293</v>
@@ -1377,13 +1438,16 @@
       <c r="F19" s="3">
         <v>30000</v>
       </c>
-      <c r="G19" s="3"/>
+      <c r="G19" s="3" cm="1">
+        <f t="array" ref="G19">Discount(E19, F19)</f>
+        <v>0</v>
+      </c>
       <c r="H19" s="4">
         <f t="shared" si="0"/>
         <v>300000</v>
       </c>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" s="1">
         <f t="shared" si="1"/>
         <v>11294</v>
@@ -1400,13 +1464,16 @@
       <c r="F20" s="3">
         <v>30000</v>
       </c>
-      <c r="G20" s="3"/>
+      <c r="G20" s="3" cm="1">
+        <f t="array" ref="G20">Discount(E20, F20)</f>
+        <v>0</v>
+      </c>
       <c r="H20" s="4">
         <f t="shared" si="0"/>
         <v>150000</v>
       </c>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" s="1">
         <f t="shared" si="1"/>
         <v>11295</v>
@@ -1423,13 +1490,16 @@
       <c r="F21" s="3">
         <v>26000</v>
       </c>
-      <c r="G21" s="3"/>
+      <c r="G21" s="3" cm="1">
+        <f t="array" ref="G21">Discount(E21, F21)</f>
+        <v>936000</v>
+      </c>
       <c r="H21" s="4">
         <f t="shared" si="0"/>
-        <v>4680000</v>
-      </c>
-    </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.35">
+        <v>3744000</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B22" s="1">
         <f t="shared" si="1"/>
         <v>11296</v>
@@ -1446,13 +1516,16 @@
       <c r="F22" s="3">
         <v>30000</v>
       </c>
-      <c r="G22" s="3"/>
+      <c r="G22" s="3" cm="1">
+        <f t="array" ref="G22">Discount(E22, F22)</f>
+        <v>0</v>
+      </c>
       <c r="H22" s="4">
         <f t="shared" si="0"/>
         <v>150000</v>
       </c>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B23" s="1">
         <f t="shared" si="1"/>
         <v>11297</v>
@@ -1469,10 +1542,13 @@
       <c r="F23" s="3">
         <v>35000</v>
       </c>
-      <c r="G23" s="3"/>
+      <c r="G23" s="3" cm="1">
+        <f t="array" ref="G23">Discount(E23, F23)</f>
+        <v>1750000</v>
+      </c>
       <c r="H23" s="4">
         <f t="shared" si="0"/>
-        <v>8750000</v>
+        <v>7000000</v>
       </c>
     </row>
   </sheetData>
@@ -1484,16 +1560,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52FE34F6-6198-3443-B91E-0337678D12FE}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="B2:H23"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
-    <col min="2" max="2" width="9.33203125" customWidth="1"/>
+    <col min="2" max="2" width="9.375" customWidth="1"/>
     <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.6640625" customWidth="1"/>
+    <col min="5" max="5" width="9.625" customWidth="1"/>
     <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="2" spans="2:8" ht="21" x14ac:dyDescent="0.35">
       <c r="B2" s="5" t="s">
         <v>37</v>
       </c>
@@ -1504,12 +1580,12 @@
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="7" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="8" t="s">
         <v>2</v>
       </c>
@@ -1532,7 +1608,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="1">
         <v>11280</v>
       </c>
@@ -1554,7 +1630,7 @@
         <v>450000</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="1">
         <f>B6+1</f>
         <v>11281</v>
@@ -1577,7 +1653,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="1">
         <f t="shared" ref="B8:B23" si="1">B7+1</f>
         <v>11282</v>
@@ -1600,7 +1676,7 @@
         <v>4200000</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="1">
         <f t="shared" si="1"/>
         <v>11283</v>
@@ -1623,7 +1699,7 @@
         <v>360000</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="1">
         <f t="shared" si="1"/>
         <v>11284</v>
@@ -1646,7 +1722,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="1">
         <f t="shared" si="1"/>
         <v>11285</v>
@@ -1669,7 +1745,7 @@
         <v>520000</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" s="1">
         <f t="shared" si="1"/>
         <v>11286</v>
@@ -1692,7 +1768,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="1">
         <f t="shared" si="1"/>
         <v>11287</v>
@@ -1715,7 +1791,7 @@
         <v>175000</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" s="1">
         <f t="shared" si="1"/>
         <v>11288</v>
@@ -1738,7 +1814,7 @@
         <v>2400000</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="1">
         <f t="shared" si="1"/>
         <v>11289</v>
@@ -1761,7 +1837,7 @@
         <v>2600000</v>
       </c>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16" s="1">
         <f t="shared" si="1"/>
         <v>11290</v>
@@ -1784,7 +1860,7 @@
         <v>700000</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="1">
         <f t="shared" si="1"/>
         <v>11291</v>
@@ -1807,7 +1883,7 @@
         <v>1000000</v>
       </c>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="1">
         <f t="shared" si="1"/>
         <v>11292</v>
@@ -1830,7 +1906,7 @@
         <v>280000</v>
       </c>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="1">
         <f t="shared" si="1"/>
         <v>11293</v>
@@ -1853,7 +1929,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" s="1">
         <f t="shared" si="1"/>
         <v>11294</v>
@@ -1876,7 +1952,7 @@
         <v>150000</v>
       </c>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" s="1">
         <f t="shared" si="1"/>
         <v>11295</v>
@@ -1899,7 +1975,7 @@
         <v>4680000</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B22" s="1">
         <f t="shared" si="1"/>
         <v>11296</v>
@@ -1922,7 +1998,7 @@
         <v>150000</v>
       </c>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B23" s="1">
         <f t="shared" si="1"/>
         <v>11297</v>

</xml_diff>

<commit_message>
Added send email sub
Added a sub that sends the excel file as an attachment in an email. This creates a pop up before sending. Learned how to create variables and clear memory at the end of functions.
</commit_message>
<xml_diff>
--- a/Excel-VBA-Start.xlsx
+++ b/Excel-VBA-Start.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\belin\Documents\CMPT310_A2\VBA_Learning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F274FFE3-93FD-4BEA-8CAF-0720B47E6A09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3723135-094E-4DE2-909E-9159F11F5FFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" activeTab="2" xr2:uid="{107DEBDB-C5C3-F842-80B8-32945E357030}"/>
   </bookViews>
@@ -557,6 +557,10 @@
 <formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Button" lockText="1"/>
 </file>
 
+<file path=xl/ctrlProps/ctrlProp2.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Button" lockText="1"/>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
@@ -663,6 +667,75 @@
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:t>Clear</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+        <xdr:clientData fPrintsWithSheet="0"/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>9</xdr:col>
+          <xdr:colOff>85725</xdr:colOff>
+          <xdr:row>4</xdr:row>
+          <xdr:rowOff>28575</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>10</xdr:col>
+          <xdr:colOff>257175</xdr:colOff>
+          <xdr:row>6</xdr:row>
+          <xdr:rowOff>57150</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="3074" name="Button 2" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s3074"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-0000020C0000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln w="9525">
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="27432" rIns="27432" bIns="27432" anchor="ctr" upright="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr sz="1000"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-CA" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Calibri"/>
+                  <a:cs typeface="Calibri"/>
+                </a:rPr>
+                <a:t>Send Email</a:t>
               </a:r>
             </a:p>
           </xdr:txBody>
@@ -1784,6 +1857,28 @@
             </control>
           </mc:Choice>
         </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="3074" r:id="rId5" name="Button 2">
+              <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="[0]!SendEmail">
+                <anchor moveWithCells="1" sizeWithCells="1">
+                  <from>
+                    <xdr:col>9</xdr:col>
+                    <xdr:colOff>85725</xdr:colOff>
+                    <xdr:row>4</xdr:row>
+                    <xdr:rowOff>28575</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>10</xdr:col>
+                    <xdr:colOff>257175</xdr:colOff>
+                    <xdr:row>6</xdr:row>
+                    <xdr:rowOff>57150</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
       </controls>
     </mc:Choice>
   </mc:AlternateContent>

</xml_diff>